<commit_message>
Fix workbook corruption (overlapping column defs); freeze rows + columns
The previous styling produced overlapping <col> ranges (the original file's
multi-column defs left in place while per-column widths were added on top),
which made Excel show "We found a problem with some content." Also dropped the
cell comments (VML) as a secondary risk.

Rebuilt the styling from the clean pre-styling workbook: reset each sheet's
column definitions before applying fresh single-column widths (verified zero
overlapping <col> entries, all parts well-formed). Freeze is now rows AND
columns again — Sessions: header row + Session/Book/Chapter/Topic; Division
Questions: header row + Session/Topic/Division/Range/Title. Kept the colour
coding, borders, banding, dropdowns, 100% zoom, open-at-top view. Content
re-verified byte-identical.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
+++ b/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
@@ -325,78 +325,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Guide</author>
-  </authors>
-  <commentList>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Short scene-setting note shown to the reader before the session begins. Optional.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>One division per line.  Format:   range | title
-e.g.  Genesis 1:1-2:3 | The first creation account</t>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <t>One link per line.  Format:   Label|URL
-e.g.  ESV Genesis 1|https://...</t>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
-      <text>
-        <t>Kingdom, Salvation, or Promises (pick from the dropdown). Compound is allowed, e.g. 'Promises &amp; Kingdom'.</t>
-      </text>
-    </comment>
-    <comment ref="AL1" authorId="0" shapeId="0">
-      <text>
-        <t>study or review (dropdown). 'review' is for recap sessions like Session 12.</t>
-      </text>
-    </comment>
-    <comment ref="AM1" authorId="0" shapeId="0">
-      <text>
-        <t>Only for review sessions — the range they revisit, e.g. 2-11.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Guide</author>
-  </authors>
-  <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Reference only — not read by the website. Helps you keep your place.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Must match a line in this session's 'Passage Divisions' on the Sessions tab.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Leave a question's Prompt blank and that whole question simply won't appear.</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>Shown to the reader when they finish this division.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1390,10 +1318,10 @@
     <col width="8" customWidth="1" style="6" min="1" max="1"/>
     <col width="16" customWidth="1" style="6" min="2" max="2"/>
     <col width="9" customWidth="1" style="6" min="3" max="3"/>
-    <col width="22" customWidth="1" style="6" min="4" max="6"/>
+    <col width="22" customWidth="1" style="6" min="4" max="4"/>
     <col width="34" customWidth="1" style="6" min="5" max="5"/>
     <col width="34" customWidth="1" style="6" min="6" max="6"/>
-    <col width="32" customWidth="1" style="6" min="7" max="15"/>
+    <col width="32" customWidth="1" style="6" min="7" max="7"/>
     <col width="34" customWidth="1" style="6" min="8" max="8"/>
     <col width="30" customWidth="1" style="6" min="9" max="9"/>
     <col width="22" customWidth="1" style="6" min="10" max="10"/>
@@ -1402,21 +1330,28 @@
     <col width="26" customWidth="1" style="6" min="13" max="13"/>
     <col width="26" customWidth="1" style="6" min="14" max="14"/>
     <col width="24" customWidth="1" style="6" min="15" max="15"/>
-    <col width="18" customWidth="1" style="6" min="16" max="17"/>
+    <col width="18" customWidth="1" style="6" min="16" max="16"/>
     <col width="32" customWidth="1" style="6" min="17" max="17"/>
-    <col width="30" customWidth="1" style="6" min="18" max="20"/>
+    <col width="30" customWidth="1" style="6" min="18" max="18"/>
     <col width="30" customWidth="1" style="6" min="19" max="19"/>
     <col width="30" customWidth="1" style="6" min="20" max="20"/>
-    <col outlineLevel="1" width="13" customWidth="1" style="6" min="21" max="24"/>
+    <col width="13" customWidth="1" style="6" min="21" max="21"/>
+    <col width="26" customWidth="1" style="6" min="22" max="22"/>
+    <col width="13" customWidth="1" style="6" min="23" max="23"/>
+    <col width="26" customWidth="1" style="6" min="24" max="24"/>
     <col width="30" customWidth="1" style="6" min="25" max="25"/>
     <col width="22" customWidth="1" style="6" min="26" max="26"/>
     <col width="26" customWidth="1" style="6" min="27" max="27"/>
     <col width="22" customWidth="1" style="6" min="28" max="28"/>
-    <col width="24" customWidth="1" style="6" min="29" max="32"/>
+    <col width="24" customWidth="1" style="6" min="29" max="29"/>
     <col width="24" customWidth="1" style="6" min="30" max="30"/>
     <col width="24" customWidth="1" style="6" min="31" max="31"/>
     <col width="24" customWidth="1" style="6" min="32" max="32"/>
-    <col outlineLevel="1" width="22" customWidth="1" style="6" min="33" max="37"/>
+    <col width="22" customWidth="1" style="6" min="33" max="33"/>
+    <col width="22" customWidth="1" style="6" min="34" max="34"/>
+    <col width="22" customWidth="1" style="6" min="35" max="35"/>
+    <col width="22" customWidth="1" style="6" min="36" max="36"/>
+    <col width="22" customWidth="1" style="6" min="37" max="37"/>
     <col width="15" customWidth="1" style="6" min="38" max="38"/>
     <col width="15" customWidth="1" style="6" min="39" max="39"/>
   </cols>
@@ -3450,7 +3385,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3464,12 +3398,12 @@
   <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.5"/>
   <cols>
-    <col width="8" customWidth="1" style="6" min="1" max="3"/>
+    <col width="8" customWidth="1" style="6" min="1" max="1"/>
     <col width="22" customWidth="1" style="6" min="2" max="2"/>
     <col width="9" customWidth="1" style="6" min="3" max="3"/>
-    <col width="30" customWidth="1" style="6" min="4" max="5"/>
+    <col width="30" customWidth="1" style="6" min="4" max="4"/>
     <col width="28" customWidth="1" style="6" min="5" max="5"/>
-    <col width="30" customWidth="1" style="6" min="6" max="15"/>
+    <col width="30" customWidth="1" style="6" min="6" max="6"/>
     <col width="22" customWidth="1" style="6" min="7" max="7"/>
     <col width="32" customWidth="1" style="6" min="8" max="8"/>
     <col width="30" customWidth="1" style="6" min="9" max="9"/>
@@ -5555,7 +5489,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Recap: portal mode-switch modal to body, enlarge, anchor near top
The modal was rendered inside .rc-mode, so a transformed ancestor anchored
its fixed positioning to that element and pushed it off-screen at 100% zoom.
Portal it to document.body, top-align with a 7vh offset, and scale up the
box, title, body, and button (with mobile fallbacks) for readability.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
+++ b/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeLocal\OTOverviewAG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F752308-0BED-4EB6-BD14-26B7E1F3AC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E47CBDF-69AA-45B5-82DD-99B50FB649C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1155" uniqueCount="712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="719">
   <si>
     <t>Session #</t>
   </si>
@@ -2266,7 +2266,30 @@
     <t>The law reminds the Israelites of who God is and what He has done- that they may obey Him.</t>
   </si>
   <si>
-    <t xml:space="preserve">Notice the shift in language, especially a word in 30:1 : "WHEN". </t>
+    <t>Notice the shift in language, especially a word in 30:1 : "WHEN", signalling what follows (blessings, curses etc.) WILL happen. What is Israel's foretold future in v1-10?</t>
+  </si>
+  <si>
+    <t>The blessings AND curses will befall them. Then, they will "call to mind" God's Words, and return to Him in obedience with all their heart and soul. God Himself circumcises their hearts SO that they can love Him with all their hearts and souls. He will delight in blessing them more abundantly than their forefathers.</t>
+  </si>
+  <si>
+    <t>Look at V11-14. Why is it "Not too hard" for Israel to obey God? Do you agree?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The word is very near them - the written law, spoken and practiced in the various rituals. Yet they have to obey ALL the commandments, with their hearts as well. The big issue - this can only be done when God circumcises their hearts (Deut 30:6). </t>
+  </si>
+  <si>
+    <t>Look at Deut 30:15,19-20. What are the stakes involved in the choice Israel makes?</t>
+  </si>
+  <si>
+    <t>Life and good vs Death and evil. They should choose life - for God is their life, that they may enjoy God's covenantal promises.</t>
+  </si>
+  <si>
+    <t>Israel's disobedience is foretold. Yet God promises to circumcises their hearts, and they will ultimately obey Him with all their heart and soul, and enjoy God's blessings in full.</t>
+  </si>
+  <si>
+    <t>God has revealed all His works and His words through the law for Israel to obey, which God’s people must “do all”  for His blessings to follow; if not His curses will overwhelm them, especially through other nations. 
+Yet they could not do so due to their inability to truly love God, needing God to circumcise their hearts. 
+God foretells their failure, but also an eventual restoration of His perfect kingdom order through the circumcising of their hearts.</t>
   </si>
 </sst>
 </file>
@@ -4475,7 +4498,7 @@
         <v>270</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>271</v>
+        <v>718</v>
       </c>
       <c r="J12" s="12" t="s">
         <v>272</v>
@@ -6037,7 +6060,7 @@
       </c>
       <c r="P33" s="13"/>
     </row>
-    <row r="34" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" ht="100" x14ac:dyDescent="0.35">
       <c r="A34" s="12">
         <v>11</v>
       </c>
@@ -6057,14 +6080,26 @@
         <v>711</v>
       </c>
       <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
+      <c r="H34" s="12" t="s">
+        <v>712</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>713</v>
+      </c>
       <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
+      <c r="K34" s="12" t="s">
+        <v>714</v>
+      </c>
+      <c r="L34" s="12" t="s">
+        <v>715</v>
+      </c>
       <c r="M34" s="12"/>
-      <c r="N34" s="12"/>
-      <c r="O34" s="12"/>
+      <c r="N34" s="12" t="s">
+        <v>716</v>
+      </c>
+      <c r="O34" s="12" t="s">
+        <v>717</v>
+      </c>
       <c r="P34" s="12"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recap: Meditate-only Pentateuch Review, Visited badge, refreshed content
- Session 12 now renders Meditate-only: embeds the full Big Picture subway
  map, OT reflect questions (Salvation/Promises/Kingdom highlighted), NT
  fulfilment boxes (Tensions + John 1:16-17, Salvation-through-Christ
  click-to-reveals + summary, God's promised Kingdom), an NT reflection,
  and a sessions-2-11-style Pause & Pray. Standalone reflection timer removed.
- Meditate picker: drop per-session and overall progress rings; show a green
  "Visited" badge when any input exists (robust whole-record text check).
- Regenerate content-overrides.js from the latest Data Entry workbook
  (updated Meditate OT/NT reflect questions across sessions).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
+++ b/RECAP MODE - Data Entry USE THIS v9 (synced).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ClaudeLocal\OTOverviewAG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E47CBDF-69AA-45B5-82DD-99B50FB649C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{703E27E0-AA83-4639-8996-1918A2A26298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="719">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="733">
   <si>
     <t>Session #</t>
   </si>
@@ -895,9 +895,6 @@
 Deuteronomy 30 | Choose life and not death, Israel's future foretold</t>
   </si>
   <si>
-    <t>God has revealed all His works and His words through the law for Israel to obey, which God’s people must “do all”  for His blessings to follow; if not His curses will overwhelm them, especially through other nations. Yet they could not do so due to their inability to truly love God, needing God to circumcise their hearts. God foretells their failure, but also an eventual restoration of His perfect kingdom order through the circumcising of their hearts.</t>
-  </si>
-  <si>
     <t>Deuteronomy 30:6 - And the Lord your God will circumcise your heart and the heart of your offspring, so that you will love the Lord your God with all your heart and with all your soul, that you may live.</t>
   </si>
   <si>
@@ -914,14 +911,6 @@
   </si>
   <si>
     <t>Romans 10:5-13</t>
-  </si>
-  <si>
-    <t>Israel’s spiritual inability to full love God from the heart (Deut. 6) is no different from
-us, so Israel serves to point us to the Better Word – Christ the true fulfillment of the Word proclaimed in Deut. 30.
-For the "righteousness based in faith" (and not the law), we are to confess and believe"in our heart" that Jesus is Lord to be saved into relationship with Him.</t>
-  </si>
-  <si>
-    <t>How does today’s OT episode help your heart (or not) behold the riches we have in the gospel? Why (or why not)?</t>
   </si>
   <si>
     <t>hearts</t>
@@ -2290,6 +2279,57 @@
     <t>God has revealed all His works and His words through the law for Israel to obey, which God’s people must “do all”  for His blessings to follow; if not His curses will overwhelm them, especially through other nations. 
 Yet they could not do so due to their inability to truly love God, needing God to circumcise their hearts. 
 God foretells their failure, but also an eventual restoration of His perfect kingdom order through the circumcising of their hearts.</t>
+  </si>
+  <si>
+    <t>How does seeing God's good kingdom patterns help you appreciate Him better?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God. What are the sins God is asking you to repent of now?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How are you feeling towards God’s character and commitment to save his people? </t>
+  </si>
+  <si>
+    <t>Pause and speak to God. How confident are you in His promises? Why/Why not?</t>
+  </si>
+  <si>
+    <t>Christ is our Passover lamb. Pause and dwell on this truth - write down your feelings and thoughts.</t>
+  </si>
+  <si>
+    <t>How do you feel about who God is and how he saves?</t>
+  </si>
+  <si>
+    <t>How does seeing God's plan and goodness help me appreciate Jesus' rule better?</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Looking at our world today, what is my yearning and anticipation for God's salvation plan?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God. How am I feeling towards God's holiness?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God - What do I feel towards Jesus and Mt Zion?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God. What does my relationship with God look like?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God. How do I view my sin and its consequences in my life?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God - How do I feel towards Jesus as the gracious mediator?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God - How do I feel towards Jesus as the perfect mediator, enabling full access to God?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God - How do I feel towards Jesus as my great High Priest and perfect sacrifice?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God. Consider His love for me. Do I love Him with all my heart and soul now?</t>
+  </si>
+  <si>
+    <t>Pause and speak to God. Consider His love for me. Take time to behold all the riches we have in the gospel.</t>
   </si>
 </sst>
 </file>
@@ -2463,7 +2503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2524,6 +2564,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2875,107 +2921,107 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="21" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="20" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B5" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C5" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B6" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C6" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B7" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C7" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B8" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C8" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="20" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="20"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B11" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C11" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B12" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C12" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B13" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C13" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -2983,87 +3029,87 @@
         <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C14" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B15" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C15" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B16" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="C16" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B17" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C17" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="B18" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C18" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B19" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C19" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="B20" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C20" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B21" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C21" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -3073,232 +3119,232 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B24" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B25" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B26" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B27" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B30" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B31" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B32" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="B35" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B36" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B37" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B38" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B41" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B42" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B43" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B44" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="93" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="62" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="62" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="B56" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="B57" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="B58" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -3583,7 +3629,7 @@
         <v>67</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="F3" s="13" t="s">
         <v>68</v>
@@ -3663,8 +3709,12 @@
       <c r="AK3" s="13"/>
       <c r="AL3" s="13"/>
       <c r="AM3" s="13"/>
-      <c r="AN3" s="19"/>
-      <c r="AO3" s="19"/>
+      <c r="AN3" s="22" t="s">
+        <v>716</v>
+      </c>
+      <c r="AO3" s="22" t="s">
+        <v>722</v>
+      </c>
     </row>
     <row r="4" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="12">
@@ -3683,7 +3733,7 @@
         <v>88</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>89</v>
@@ -3719,10 +3769,10 @@
         <v>98</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="T4" s="12"/>
       <c r="U4" s="12" t="s">
@@ -3764,8 +3814,12 @@
       <c r="AK4" s="12"/>
       <c r="AL4" s="12"/>
       <c r="AM4" s="12"/>
-      <c r="AN4" s="18"/>
-      <c r="AO4" s="18"/>
+      <c r="AN4" s="23" t="s">
+        <v>717</v>
+      </c>
+      <c r="AO4" s="12" t="s">
+        <v>723</v>
+      </c>
     </row>
     <row r="5" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13">
@@ -3865,8 +3919,12 @@
       <c r="AK5" s="13"/>
       <c r="AL5" s="13"/>
       <c r="AM5" s="13"/>
-      <c r="AN5" s="19"/>
-      <c r="AO5" s="19"/>
+      <c r="AN5" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="AO5" s="13" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="6" spans="1:41" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="12">
@@ -3919,10 +3977,10 @@
         <v>143</v>
       </c>
       <c r="R6" s="12" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="T6" s="12" t="s">
         <v>144</v>
@@ -3966,8 +4024,12 @@
       <c r="AK6" s="12"/>
       <c r="AL6" s="12"/>
       <c r="AM6" s="12"/>
-      <c r="AN6" s="18"/>
-      <c r="AO6" s="18"/>
+      <c r="AN6" s="23" t="s">
+        <v>718</v>
+      </c>
+      <c r="AO6" s="23" t="s">
+        <v>719</v>
+      </c>
     </row>
     <row r="7" spans="1:41" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13">
@@ -4065,8 +4127,12 @@
       <c r="AK7" s="13"/>
       <c r="AL7" s="13"/>
       <c r="AM7" s="13"/>
-      <c r="AN7" s="19"/>
-      <c r="AO7" s="19"/>
+      <c r="AN7" s="22" t="s">
+        <v>721</v>
+      </c>
+      <c r="AO7" s="22" t="s">
+        <v>720</v>
+      </c>
     </row>
     <row r="8" spans="1:41" ht="124" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="12">
@@ -4166,8 +4232,12 @@
       <c r="AK8" s="12"/>
       <c r="AL8" s="12"/>
       <c r="AM8" s="12"/>
-      <c r="AN8" s="18"/>
-      <c r="AO8" s="18"/>
+      <c r="AN8" s="23" t="s">
+        <v>724</v>
+      </c>
+      <c r="AO8" s="23" t="s">
+        <v>725</v>
+      </c>
     </row>
     <row r="9" spans="1:41" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
@@ -4225,10 +4295,10 @@
         <v>212</v>
       </c>
       <c r="S9" s="13" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="T9" s="13" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="U9" s="13" t="s">
         <v>213</v>
@@ -4269,8 +4339,12 @@
       <c r="AK9" s="13"/>
       <c r="AL9" s="13"/>
       <c r="AM9" s="13"/>
-      <c r="AN9" s="19"/>
-      <c r="AO9" s="19"/>
+      <c r="AN9" s="22" t="s">
+        <v>726</v>
+      </c>
+      <c r="AO9" s="22" t="s">
+        <v>729</v>
+      </c>
     </row>
     <row r="10" spans="1:41" ht="170.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="12">
@@ -4370,8 +4444,12 @@
       <c r="AK10" s="12"/>
       <c r="AL10" s="12"/>
       <c r="AM10" s="12"/>
-      <c r="AN10" s="18"/>
-      <c r="AO10" s="18"/>
+      <c r="AN10" s="23" t="s">
+        <v>727</v>
+      </c>
+      <c r="AO10" s="23" t="s">
+        <v>728</v>
+      </c>
     </row>
     <row r="11" spans="1:41" ht="201.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
@@ -4427,7 +4505,7 @@
         <v>257</v>
       </c>
       <c r="S11" s="13" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="T11" s="13"/>
       <c r="U11" s="13" t="s">
@@ -4469,8 +4547,12 @@
       <c r="AK11" s="13"/>
       <c r="AL11" s="13"/>
       <c r="AM11" s="13"/>
-      <c r="AN11" s="19"/>
-      <c r="AO11" s="19"/>
+      <c r="AN11" s="22" t="s">
+        <v>724</v>
+      </c>
+      <c r="AO11" s="22" t="s">
+        <v>730</v>
+      </c>
     </row>
     <row r="12" spans="1:41" ht="263.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="12">
@@ -4498,61 +4580,61 @@
         <v>270</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="J12" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="K12" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="K12" s="12" t="s">
+      <c r="L12" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="M12" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="N12" s="12" t="s">
         <v>274</v>
       </c>
-      <c r="M12" s="12" t="s">
-        <v>274</v>
-      </c>
-      <c r="N12" s="12" t="s">
+      <c r="O12" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="O12" s="12" t="s">
+      <c r="P12" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="P12" s="12" t="s">
-        <v>277</v>
-      </c>
       <c r="Q12" s="12" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="R12" s="12" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="T12" s="12"/>
       <c r="U12" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="V12" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="W12" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="X12" s="12" t="s">
         <v>280</v>
-      </c>
-      <c r="V12" s="12" t="s">
-        <v>281</v>
-      </c>
-      <c r="W12" s="12" t="s">
-        <v>282</v>
-      </c>
-      <c r="X12" s="12" t="s">
-        <v>283</v>
       </c>
       <c r="Y12" s="12"/>
       <c r="Z12" s="12" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="AA12" s="12"/>
       <c r="AB12" s="12" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="AC12" s="12" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="AD12" s="12" t="s">
         <v>61</v>
@@ -4570,32 +4652,36 @@
       <c r="AK12" s="12"/>
       <c r="AL12" s="12"/>
       <c r="AM12" s="12"/>
-      <c r="AN12" s="18"/>
-      <c r="AO12" s="18"/>
+      <c r="AN12" s="23" t="s">
+        <v>731</v>
+      </c>
+      <c r="AO12" s="23" t="s">
+        <v>732</v>
+      </c>
     </row>
     <row r="13" spans="1:41" ht="87.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="F13" s="13" t="s">
         <v>288</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>290</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>291</v>
       </c>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
       <c r="I13" s="13" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="J13" s="13"/>
       <c r="K13" s="13"/>
@@ -4609,10 +4695,10 @@
       <c r="S13" s="13"/>
       <c r="T13" s="13"/>
       <c r="U13" s="13" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="V13" s="13" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="W13" s="13"/>
       <c r="X13" s="13"/>
@@ -4621,7 +4707,7 @@
       <c r="AA13" s="13"/>
       <c r="AB13" s="13"/>
       <c r="AC13" s="13" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="AD13" s="13" t="s">
         <v>61</v>
@@ -4641,7 +4727,7 @@
         <v>64</v>
       </c>
       <c r="AM13" s="13" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="AN13" s="19"/>
       <c r="AO13" s="19"/>
@@ -4689,49 +4775,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="14" t="s">
         <v>404</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="I1" s="15" t="s">
         <v>405</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="J1" s="15" t="s">
         <v>406</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="K1" s="15" t="s">
         <v>407</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="L1" s="16" t="s">
         <v>408</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="M1" s="16" t="s">
         <v>409</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="N1" s="16" t="s">
         <v>410</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="O1" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="P1" s="11" t="s">
         <v>412</v>
-      </c>
-      <c r="N1" s="16" t="s">
-        <v>413</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>414</v>
-      </c>
-      <c r="P1" s="11" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -4748,7 +4834,7 @@
         <v>49</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
@@ -4776,7 +4862,7 @@
         <v>50</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
@@ -4804,7 +4890,7 @@
         <v>51</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
@@ -4829,40 +4915,40 @@
         <v>1</v>
       </c>
       <c r="D5" s="13" t="s">
+        <v>416</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>417</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>418</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>419</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="H5" s="13" t="s">
         <v>420</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="I5" s="13" t="s">
+        <v>689</v>
+      </c>
+      <c r="J5" s="13" t="s">
         <v>421</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="K5" s="13" t="s">
         <v>422</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="L5" s="13" t="s">
         <v>423</v>
       </c>
-      <c r="I5" s="13" t="s">
-        <v>692</v>
-      </c>
-      <c r="J5" s="13" t="s">
+      <c r="M5" s="13" t="s">
         <v>424</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="N5" s="13" t="s">
         <v>425</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="O5" s="13" t="s">
         <v>426</v>
-      </c>
-      <c r="M5" s="13" t="s">
-        <v>427</v>
-      </c>
-      <c r="N5" s="13" t="s">
-        <v>428</v>
-      </c>
-      <c r="O5" s="13" t="s">
-        <v>429</v>
       </c>
       <c r="P5" s="13"/>
     </row>
@@ -4877,40 +4963,40 @@
         <v>2</v>
       </c>
       <c r="D6" s="12" t="s">
+        <v>427</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>428</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>429</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>430</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="H6" s="12" t="s">
         <v>431</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>432</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="J6" s="12" t="s">
         <v>433</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="K6" s="12" t="s">
         <v>434</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="L6" s="12" t="s">
         <v>435</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="M6" s="12" t="s">
         <v>436</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="N6" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="O6" s="12" t="s">
         <v>438</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>439</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>440</v>
-      </c>
-      <c r="O6" s="12" t="s">
-        <v>441</v>
       </c>
       <c r="P6" s="12"/>
     </row>
@@ -4925,32 +5011,32 @@
         <v>1</v>
       </c>
       <c r="D7" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>440</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>441</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>442</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>443</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>444</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>445</v>
       </c>
       <c r="H7" s="13"/>
       <c r="I7" s="13" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="L7" s="13"/>
       <c r="M7" s="13"/>
       <c r="N7" s="13"/>
       <c r="O7" s="13" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="P7" s="13"/>
     </row>
@@ -4965,34 +5051,34 @@
         <v>2</v>
       </c>
       <c r="D8" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>447</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="G8" s="12" t="s">
         <v>449</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="H8" s="12" t="s">
         <v>450</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="I8" s="12" t="s">
         <v>451</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="J8" s="12" t="s">
         <v>452</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="K8" s="12" t="s">
         <v>453</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>454</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>455</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>456</v>
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
       <c r="N8" s="12"/>
       <c r="O8" s="12" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="P8" s="12"/>
     </row>
@@ -5007,28 +5093,28 @@
         <v>3</v>
       </c>
       <c r="D9" s="13" t="s">
+        <v>455</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>456</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>457</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>458</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="H9" s="13" t="s">
         <v>459</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>460</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>461</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>462</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>463</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>464</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>465</v>
       </c>
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
@@ -5047,36 +5133,36 @@
         <v>1</v>
       </c>
       <c r="D10" s="12" t="s">
+        <v>463</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>464</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>465</v>
+      </c>
+      <c r="G10" s="12" t="s">
         <v>466</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="H10" s="12" t="s">
         <v>467</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="I10" s="12" t="s">
         <v>468</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>469</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>470</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>471</v>
       </c>
       <c r="J10" s="12"/>
       <c r="K10" s="12" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="M10" s="12"/>
       <c r="N10" s="12" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="O10" s="12" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="P10" s="12"/>
     </row>
@@ -5091,40 +5177,40 @@
         <v>2</v>
       </c>
       <c r="D11" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>474</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>475</v>
+      </c>
+      <c r="G11" s="13" t="s">
         <v>476</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="H11" s="13" t="s">
         <v>477</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="I11" s="13" t="s">
         <v>478</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="J11" s="13" t="s">
         <v>479</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="K11" s="13" t="s">
         <v>480</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="L11" s="13" t="s">
         <v>481</v>
       </c>
-      <c r="J11" s="13" t="s">
+      <c r="M11" s="13" t="s">
         <v>482</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="N11" s="13" t="s">
         <v>483</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="O11" s="13" t="s">
         <v>484</v>
-      </c>
-      <c r="M11" s="13" t="s">
-        <v>485</v>
-      </c>
-      <c r="N11" s="13" t="s">
-        <v>486</v>
-      </c>
-      <c r="O11" s="13" t="s">
-        <v>487</v>
       </c>
       <c r="P11" s="13"/>
     </row>
@@ -5139,40 +5225,40 @@
         <v>3</v>
       </c>
       <c r="D12" s="12" t="s">
+        <v>485</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>486</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>488</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="H12" s="12" t="s">
         <v>489</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="I12" s="12" t="s">
         <v>490</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="J12" s="12" t="s">
         <v>491</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="K12" s="12" t="s">
         <v>492</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="L12" s="12" t="s">
         <v>493</v>
       </c>
-      <c r="J12" s="12" t="s">
+      <c r="M12" s="12" t="s">
         <v>494</v>
       </c>
-      <c r="K12" s="12" t="s">
+      <c r="N12" s="12" t="s">
         <v>495</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="O12" s="12" t="s">
         <v>496</v>
-      </c>
-      <c r="M12" s="12" t="s">
-        <v>497</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>498</v>
-      </c>
-      <c r="O12" s="12" t="s">
-        <v>499</v>
       </c>
       <c r="P12" s="12"/>
     </row>
@@ -5187,34 +5273,34 @@
         <v>1</v>
       </c>
       <c r="D13" s="13" t="s">
+        <v>497</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>499</v>
+      </c>
+      <c r="G13" s="13" t="s">
         <v>500</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="H13" s="13" t="s">
         <v>501</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="I13" s="13" t="s">
         <v>502</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="J13" s="13" t="s">
         <v>503</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="K13" s="13" t="s">
         <v>504</v>
-      </c>
-      <c r="I13" s="13" t="s">
-        <v>505</v>
-      </c>
-      <c r="J13" s="13" t="s">
-        <v>506</v>
-      </c>
-      <c r="K13" s="13" t="s">
-        <v>507</v>
       </c>
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
       <c r="O13" s="13" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="P13" s="13"/>
     </row>
@@ -5229,34 +5315,34 @@
         <v>2</v>
       </c>
       <c r="D14" s="12" t="s">
+        <v>506</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>507</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>508</v>
+      </c>
+      <c r="G14" s="12" t="s">
         <v>509</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="H14" s="12" t="s">
         <v>510</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="I14" s="12" t="s">
         <v>511</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="J14" s="12" t="s">
         <v>512</v>
       </c>
-      <c r="H14" s="12" t="s">
+      <c r="K14" s="12" t="s">
         <v>513</v>
-      </c>
-      <c r="I14" s="12" t="s">
-        <v>514</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>515</v>
-      </c>
-      <c r="K14" s="12" t="s">
-        <v>516</v>
       </c>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
       <c r="O14" s="12" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="P14" s="12"/>
     </row>
@@ -5271,32 +5357,32 @@
         <v>3</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="13" t="s">
+        <v>518</v>
+      </c>
+      <c r="I15" s="13" t="s">
+        <v>519</v>
+      </c>
+      <c r="J15" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="K15" s="13" t="s">
         <v>521</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>522</v>
-      </c>
-      <c r="J15" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>524</v>
       </c>
       <c r="L15" s="13"/>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
       <c r="O15" s="13" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="P15" s="13"/>
     </row>
@@ -5311,38 +5397,38 @@
         <v>1</v>
       </c>
       <c r="D16" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>524</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="G16" s="12" t="s">
         <v>526</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="H16" s="12" t="s">
         <v>527</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="I16" s="12" t="s">
         <v>528</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>529</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>530</v>
-      </c>
-      <c r="I16" s="12" t="s">
-        <v>531</v>
       </c>
       <c r="J16" s="12"/>
       <c r="K16" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="L16" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="M16" s="12" t="s">
+        <v>531</v>
+      </c>
+      <c r="N16" s="12" t="s">
         <v>532</v>
       </c>
-      <c r="L16" s="12" t="s">
+      <c r="O16" s="12" t="s">
         <v>533</v>
-      </c>
-      <c r="M16" s="12" t="s">
-        <v>534</v>
-      </c>
-      <c r="N16" s="12" t="s">
-        <v>535</v>
-      </c>
-      <c r="O16" s="12" t="s">
-        <v>536</v>
       </c>
       <c r="P16" s="12"/>
     </row>
@@ -5357,19 +5443,19 @@
         <v>2</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>153</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
@@ -5378,7 +5464,7 @@
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
       <c r="O17" s="13" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="P17" s="13"/>
     </row>
@@ -5393,40 +5479,40 @@
         <v>3</v>
       </c>
       <c r="D18" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>540</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>541</v>
+      </c>
+      <c r="G18" s="12" t="s">
         <v>542</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="H18" s="12" t="s">
         <v>543</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="I18" s="12" t="s">
         <v>544</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="J18" s="12" t="s">
         <v>545</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="K18" s="12" t="s">
         <v>546</v>
       </c>
-      <c r="I18" s="12" t="s">
+      <c r="L18" s="12" t="s">
         <v>547</v>
       </c>
-      <c r="J18" s="12" t="s">
+      <c r="M18" s="12" t="s">
         <v>548</v>
       </c>
-      <c r="K18" s="12" t="s">
+      <c r="N18" s="12" t="s">
         <v>549</v>
       </c>
-      <c r="L18" s="12" t="s">
+      <c r="O18" s="12" t="s">
         <v>550</v>
-      </c>
-      <c r="M18" s="12" t="s">
-        <v>551</v>
-      </c>
-      <c r="N18" s="12" t="s">
-        <v>552</v>
-      </c>
-      <c r="O18" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="P18" s="12"/>
     </row>
@@ -5441,40 +5527,40 @@
         <v>1</v>
       </c>
       <c r="D19" s="13" t="s">
+        <v>551</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>552</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="G19" s="13" t="s">
         <v>554</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="H19" s="13" t="s">
         <v>555</v>
       </c>
-      <c r="F19" s="13" t="s">
+      <c r="I19" s="13" t="s">
         <v>556</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="J19" s="13" t="s">
         <v>557</v>
       </c>
-      <c r="H19" s="13" t="s">
+      <c r="K19" s="13" t="s">
         <v>558</v>
       </c>
-      <c r="I19" s="13" t="s">
+      <c r="L19" s="13" t="s">
         <v>559</v>
       </c>
-      <c r="J19" s="13" t="s">
+      <c r="M19" s="13" t="s">
         <v>560</v>
       </c>
-      <c r="K19" s="13" t="s">
+      <c r="N19" s="13" t="s">
         <v>561</v>
       </c>
-      <c r="L19" s="13" t="s">
+      <c r="O19" s="13" t="s">
         <v>562</v>
-      </c>
-      <c r="M19" s="13" t="s">
-        <v>563</v>
-      </c>
-      <c r="N19" s="13" t="s">
-        <v>564</v>
-      </c>
-      <c r="O19" s="13" t="s">
-        <v>565</v>
       </c>
       <c r="P19" s="13"/>
     </row>
@@ -5489,32 +5575,32 @@
         <v>2</v>
       </c>
       <c r="D20" s="12" t="s">
+        <v>563</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>565</v>
+      </c>
+      <c r="G20" s="12" t="s">
         <v>566</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="H20" s="12" t="s">
         <v>567</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="I20" s="12" t="s">
         <v>568</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>569</v>
-      </c>
-      <c r="H20" s="12" t="s">
-        <v>570</v>
-      </c>
-      <c r="I20" s="12" t="s">
-        <v>571</v>
       </c>
       <c r="J20" s="12"/>
       <c r="K20" s="12" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="L20" s="12"/>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
       <c r="O20" s="12" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="P20" s="12"/>
     </row>
@@ -5529,34 +5615,34 @@
         <v>3</v>
       </c>
       <c r="D21" s="13" t="s">
+        <v>571</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>572</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>573</v>
+      </c>
+      <c r="G21" s="13" t="s">
         <v>574</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="H21" s="13" t="s">
         <v>575</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="I21" s="13" t="s">
         <v>576</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="J21" s="13" t="s">
         <v>577</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="K21" s="13" t="s">
         <v>578</v>
-      </c>
-      <c r="I21" s="13" t="s">
-        <v>579</v>
-      </c>
-      <c r="J21" s="13" t="s">
-        <v>580</v>
-      </c>
-      <c r="K21" s="13" t="s">
-        <v>581</v>
       </c>
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
       <c r="O21" s="13" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="P21" s="13"/>
     </row>
@@ -5571,19 +5657,19 @@
         <v>4</v>
       </c>
       <c r="D22" s="12" t="s">
+        <v>580</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>581</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>582</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>583</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="H22" s="12" t="s">
         <v>584</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>585</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>586</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>587</v>
       </c>
       <c r="I22" s="12"/>
       <c r="J22" s="12"/>
@@ -5592,7 +5678,7 @@
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
       <c r="O22" s="12" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="P22" s="12"/>
     </row>
@@ -5607,34 +5693,34 @@
         <v>1</v>
       </c>
       <c r="D23" s="13" t="s">
+        <v>586</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>587</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>588</v>
+      </c>
+      <c r="G23" s="13" t="s">
         <v>589</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="H23" s="13" t="s">
         <v>590</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="I23" s="13" t="s">
         <v>591</v>
       </c>
-      <c r="G23" s="13" t="s">
+      <c r="J23" s="13" t="s">
         <v>592</v>
       </c>
-      <c r="H23" s="13" t="s">
+      <c r="K23" s="13" t="s">
         <v>593</v>
-      </c>
-      <c r="I23" s="13" t="s">
-        <v>594</v>
-      </c>
-      <c r="J23" s="13" t="s">
-        <v>595</v>
-      </c>
-      <c r="K23" s="13" t="s">
-        <v>596</v>
       </c>
       <c r="L23" s="13"/>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
       <c r="O23" s="13" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="P23" s="13"/>
     </row>
@@ -5649,40 +5735,40 @@
         <v>2</v>
       </c>
       <c r="D24" s="12" t="s">
+        <v>595</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>596</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>597</v>
+      </c>
+      <c r="G24" s="12" t="s">
         <v>598</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="H24" s="12" t="s">
         <v>599</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="I24" s="12" t="s">
         <v>600</v>
       </c>
-      <c r="G24" s="12" t="s">
+      <c r="J24" s="12" t="s">
         <v>601</v>
       </c>
-      <c r="H24" s="12" t="s">
+      <c r="K24" s="12" t="s">
         <v>602</v>
       </c>
-      <c r="I24" s="12" t="s">
+      <c r="L24" s="12" t="s">
         <v>603</v>
       </c>
-      <c r="J24" s="12" t="s">
+      <c r="M24" s="12" t="s">
         <v>604</v>
       </c>
-      <c r="K24" s="12" t="s">
+      <c r="N24" s="12" t="s">
         <v>605</v>
       </c>
-      <c r="L24" s="12" t="s">
+      <c r="O24" s="12" t="s">
         <v>606</v>
-      </c>
-      <c r="M24" s="12" t="s">
-        <v>607</v>
-      </c>
-      <c r="N24" s="12" t="s">
-        <v>608</v>
-      </c>
-      <c r="O24" s="12" t="s">
-        <v>609</v>
       </c>
       <c r="P24" s="12"/>
     </row>
@@ -5697,19 +5783,19 @@
         <v>3</v>
       </c>
       <c r="D25" s="13" t="s">
+        <v>607</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>608</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>609</v>
+      </c>
+      <c r="G25" s="13" t="s">
         <v>610</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="H25" s="13" t="s">
         <v>611</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>612</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>613</v>
-      </c>
-      <c r="H25" s="13" t="s">
-        <v>614</v>
       </c>
       <c r="I25" s="13"/>
       <c r="J25" s="13"/>
@@ -5718,7 +5804,7 @@
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
       <c r="O25" s="13" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="P25" s="13"/>
     </row>
@@ -5733,40 +5819,40 @@
         <v>1</v>
       </c>
       <c r="D26" s="12" t="s">
+        <v>613</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>614</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>615</v>
+      </c>
+      <c r="G26" s="12" t="s">
         <v>616</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="H26" s="12" t="s">
         <v>617</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="I26" s="12" t="s">
         <v>618</v>
       </c>
-      <c r="G26" s="12" t="s">
+      <c r="J26" s="12" t="s">
         <v>619</v>
       </c>
-      <c r="H26" s="12" t="s">
+      <c r="K26" s="12" t="s">
         <v>620</v>
       </c>
-      <c r="I26" s="12" t="s">
+      <c r="L26" s="12" t="s">
         <v>621</v>
       </c>
-      <c r="J26" s="12" t="s">
+      <c r="M26" s="12" t="s">
         <v>622</v>
       </c>
-      <c r="K26" s="12" t="s">
+      <c r="N26" s="12" t="s">
         <v>623</v>
       </c>
-      <c r="L26" s="12" t="s">
+      <c r="O26" s="12" t="s">
         <v>624</v>
-      </c>
-      <c r="M26" s="12" t="s">
-        <v>625</v>
-      </c>
-      <c r="N26" s="12" t="s">
-        <v>626</v>
-      </c>
-      <c r="O26" s="12" t="s">
-        <v>627</v>
       </c>
       <c r="P26" s="12"/>
     </row>
@@ -5781,19 +5867,19 @@
         <v>2</v>
       </c>
       <c r="D27" s="13" t="s">
+        <v>625</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>626</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>627</v>
+      </c>
+      <c r="G27" s="13" t="s">
         <v>628</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="H27" s="13" t="s">
         <v>629</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>630</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>631</v>
-      </c>
-      <c r="H27" s="13" t="s">
-        <v>632</v>
       </c>
       <c r="I27" s="13"/>
       <c r="J27" s="13"/>
@@ -5802,7 +5888,7 @@
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
       <c r="O27" s="13" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="P27" s="13"/>
     </row>
@@ -5817,34 +5903,34 @@
         <v>3</v>
       </c>
       <c r="D28" s="12" t="s">
+        <v>631</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>632</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>633</v>
+      </c>
+      <c r="G28" s="12" t="s">
         <v>634</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="H28" s="12" t="s">
         <v>635</v>
       </c>
-      <c r="F28" s="12" t="s">
+      <c r="I28" s="12" t="s">
         <v>636</v>
       </c>
-      <c r="G28" s="12" t="s">
+      <c r="J28" s="12" t="s">
         <v>637</v>
       </c>
-      <c r="H28" s="12" t="s">
+      <c r="K28" s="12" t="s">
         <v>638</v>
-      </c>
-      <c r="I28" s="12" t="s">
-        <v>639</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>640</v>
-      </c>
-      <c r="K28" s="12" t="s">
-        <v>641</v>
       </c>
       <c r="L28" s="12"/>
       <c r="M28" s="12"/>
       <c r="N28" s="12"/>
       <c r="O28" s="12" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="P28" s="12"/>
     </row>
@@ -5859,38 +5945,38 @@
         <v>1</v>
       </c>
       <c r="D29" s="13" t="s">
+        <v>640</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>641</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>642</v>
+      </c>
+      <c r="G29" s="13" t="s">
         <v>643</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="H29" s="13" t="s">
         <v>644</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="I29" s="13" t="s">
         <v>645</v>
       </c>
-      <c r="G29" s="13" t="s">
+      <c r="J29" s="13" t="s">
         <v>646</v>
       </c>
-      <c r="H29" s="13" t="s">
+      <c r="K29" s="13" t="s">
         <v>647</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="L29" s="13" t="s">
         <v>648</v>
-      </c>
-      <c r="J29" s="13" t="s">
-        <v>649</v>
-      </c>
-      <c r="K29" s="13" t="s">
-        <v>650</v>
-      </c>
-      <c r="L29" s="13" t="s">
-        <v>651</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="O29" s="13" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="P29" s="13"/>
     </row>
@@ -5905,34 +5991,34 @@
         <v>2</v>
       </c>
       <c r="D30" s="12" t="s">
+        <v>651</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>653</v>
+      </c>
+      <c r="G30" s="12" t="s">
         <v>654</v>
       </c>
-      <c r="E30" s="12" t="s">
+      <c r="H30" s="12" t="s">
         <v>655</v>
       </c>
-      <c r="F30" s="12" t="s">
+      <c r="I30" s="12" t="s">
         <v>656</v>
       </c>
-      <c r="G30" s="12" t="s">
+      <c r="J30" s="12" t="s">
         <v>657</v>
       </c>
-      <c r="H30" s="12" t="s">
+      <c r="K30" s="12" t="s">
         <v>658</v>
-      </c>
-      <c r="I30" s="12" t="s">
-        <v>659</v>
-      </c>
-      <c r="J30" s="12" t="s">
-        <v>660</v>
-      </c>
-      <c r="K30" s="12" t="s">
-        <v>661</v>
       </c>
       <c r="L30" s="12"/>
       <c r="M30" s="12"/>
       <c r="N30" s="12"/>
       <c r="O30" s="12" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="P30" s="12"/>
     </row>
@@ -5947,19 +6033,19 @@
         <v>3</v>
       </c>
       <c r="D31" s="13" t="s">
+        <v>660</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>661</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>662</v>
+      </c>
+      <c r="G31" s="13" t="s">
         <v>663</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="H31" s="13" t="s">
         <v>664</v>
-      </c>
-      <c r="F31" s="13" t="s">
-        <v>665</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>666</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>667</v>
       </c>
       <c r="I31" s="13"/>
       <c r="J31" s="13"/>
@@ -5968,7 +6054,7 @@
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
       <c r="O31" s="13" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="P31" s="13"/>
     </row>
@@ -5983,38 +6069,38 @@
         <v>1</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="12" t="s">
+        <v>669</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>670</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>671</v>
+      </c>
+      <c r="K32" s="12" t="s">
         <v>672</v>
       </c>
-      <c r="I32" s="12" t="s">
+      <c r="L32" s="12" t="s">
         <v>673</v>
       </c>
-      <c r="J32" s="12" t="s">
+      <c r="M32" s="12" t="s">
         <v>674</v>
       </c>
-      <c r="K32" s="12" t="s">
+      <c r="N32" s="12" t="s">
         <v>675</v>
       </c>
-      <c r="L32" s="12" t="s">
-        <v>676</v>
-      </c>
-      <c r="M32" s="12" t="s">
-        <v>677</v>
-      </c>
-      <c r="N32" s="12" t="s">
-        <v>678</v>
-      </c>
       <c r="O32" s="12" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="P32" s="12"/>
     </row>
@@ -6029,34 +6115,34 @@
         <v>2</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="G33" s="13"/>
       <c r="H33" s="13" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="I33" s="13" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="J33" s="13"/>
       <c r="K33" s="13" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="L33" s="13" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="O33" s="13" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="P33" s="13"/>
     </row>
@@ -6071,34 +6157,34 @@
         <v>3</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="G34" s="12"/>
       <c r="H34" s="12" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="J34" s="12"/>
       <c r="K34" s="12" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M34" s="12"/>
       <c r="N34" s="12" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="O34" s="12" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="P34" s="12"/>
     </row>
@@ -6126,13 +6212,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -6140,10 +6226,10 @@
         <v>2</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="D2" s="12"/>
     </row>
@@ -6152,10 +6238,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="D3" s="13"/>
     </row>

</xml_diff>